<commit_message>
commiting the reports and screenshots
</commit_message>
<xml_diff>
--- a/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
+++ b/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d74e56779d8c9e49/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\git\repository3\MakeMyTrip_Sprint\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{C83AB80F-2C5A-4B3A-B654-732051A62456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A64F945-7A11-4CA3-871C-39A085A6E1F7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43A8ACA-1F2D-44D0-BD26-1AC13B312647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="3" activeTab="4" xr2:uid="{AE859187-6724-4D77-AF72-93B2659ED249}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE859187-6724-4D77-AF72-93B2659ED249}"/>
   </bookViews>
   <sheets>
     <sheet name="Train" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="55">
   <si>
     <t>Source</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Chennai</t>
   </si>
   <si>
-    <t>Madurai</t>
-  </si>
-  <si>
     <t>Sleeper</t>
   </si>
   <si>
@@ -200,6 +197,12 @@
   </si>
   <si>
     <t>Jul</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Salem</t>
   </si>
 </sst>
 </file>
@@ -251,11 +254,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -571,13 +574,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42C36B47-3263-42EC-9348-FE092B284D98}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -585,42 +588,48 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3">
-        <v>46137</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -635,38 +644,38 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
         <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -685,186 +694,186 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
-      </c>
-      <c r="G1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
         <v>27</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>28</v>
-      </c>
-      <c r="C2" t="s">
-        <v>29</v>
       </c>
       <c r="D2">
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F2">
         <v>1997</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
         <v>32</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>33</v>
-      </c>
-      <c r="C3" t="s">
-        <v>34</v>
       </c>
       <c r="D3">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F3">
         <v>1998</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" t="s">
         <v>36</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>37</v>
-      </c>
-      <c r="C4" t="s">
-        <v>38</v>
       </c>
       <c r="D4">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F4">
         <v>1999</v>
       </c>
       <c r="G4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>41</v>
-      </c>
-      <c r="C5" t="s">
-        <v>42</v>
       </c>
       <c r="D5">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F5">
         <v>2000</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" t="s">
         <v>44</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>45</v>
-      </c>
-      <c r="C6" t="s">
-        <v>46</v>
       </c>
       <c r="D6">
         <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F6">
         <v>2001</v>
       </c>
       <c r="G6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
         <v>48</v>
       </c>
-      <c r="B7" t="s">
-        <v>49</v>
-      </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D7">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F7">
         <v>2002</v>
       </c>
       <c r="G7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" t="s">
         <v>51</v>
       </c>
-      <c r="B8" t="s">
-        <v>52</v>
-      </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D8">
         <v>17</v>
       </c>
       <c r="E8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F8">
         <v>2003</v>
       </c>
       <c r="G8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -879,71 +888,71 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>25</v>
-      </c>
-      <c r="G1" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="s">
         <v>27</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>28</v>
-      </c>
-      <c r="C2" t="s">
-        <v>29</v>
       </c>
       <c r="D2">
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F2">
         <v>1997</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" t="s">
         <v>32</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>33</v>
-      </c>
-      <c r="C3" t="s">
-        <v>34</v>
       </c>
       <c r="D3">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F3">
         <v>1998</v>
       </c>
       <c r="G3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -958,38 +967,38 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
         <v>13</v>
-      </c>
-      <c r="B1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="3"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="B4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
feat(train): add new feature files, step definitions, and update Reports
</commit_message>
<xml_diff>
--- a/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
+++ b/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\git\repository3\MakeMyTrip_Sprint\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43A8ACA-1F2D-44D0-BD26-1AC13B312647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC11D9B-7D99-43E2-9C10-FA42B6F6FCE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE859187-6724-4D77-AF72-93B2659ED249}"/>
   </bookViews>
@@ -67,12 +67,6 @@
     <t>Sleeper</t>
   </si>
   <si>
-    <t>06 AM - 12 PM</t>
-  </si>
-  <si>
-    <t>12 PM - 06 PM</t>
-  </si>
-  <si>
     <t>Superfast</t>
   </si>
   <si>
@@ -203,6 +197,12 @@
   </si>
   <si>
     <t>Salem</t>
+  </si>
+  <si>
+    <t>6 AM - 12 PM</t>
+  </si>
+  <si>
+    <t>12 PM - 6 PM</t>
   </si>
 </sst>
 </file>
@@ -254,11 +254,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -578,6 +578,9 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="9.109375" customWidth="1"/>
+    <col min="6" max="6" width="21.5546875" customWidth="1"/>
+    <col min="7" max="7" width="20.109375" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -588,7 +591,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -611,28 +614,33 @@
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>53</v>
+        <v>44</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>11</v>
-      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G19" xr:uid="{54DE1FC2-7873-4FF0-9E14-1AE5979033BC}">
+      <formula1>"12am - 6am,6am - 12pm,12pm - 6pm,6pm - 12am"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -644,38 +652,38 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="3"/>
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="3"/>
+        <v>14</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3"/>
+        <v>16</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -694,186 +702,186 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
       </c>
       <c r="D2">
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F2">
         <v>1997</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
         <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>33</v>
       </c>
       <c r="D3">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F3">
         <v>1998</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" t="s">
         <v>35</v>
-      </c>
-      <c r="B4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" t="s">
-        <v>37</v>
       </c>
       <c r="D4">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F4">
         <v>1999</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" t="s">
         <v>39</v>
-      </c>
-      <c r="B5" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
       </c>
       <c r="D5">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F5">
         <v>2000</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
         <v>43</v>
-      </c>
-      <c r="B6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" t="s">
-        <v>45</v>
       </c>
       <c r="D6">
         <v>15</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F6">
         <v>2001</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D7">
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F7">
         <v>2002</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D8">
         <v>17</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F8">
         <v>2003</v>
       </c>
       <c r="G8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -888,71 +896,71 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>23</v>
-      </c>
-      <c r="F1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" t="s">
         <v>26</v>
-      </c>
-      <c r="B2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C2" t="s">
-        <v>28</v>
       </c>
       <c r="D2">
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F2">
         <v>1997</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
         <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>33</v>
       </c>
       <c r="D3">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F3">
         <v>1998</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -967,38 +975,38 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="3"/>
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="3"/>
+        <v>14</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="3"/>
+        <v>16</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Commiting the updated excel file
</commit_message>
<xml_diff>
--- a/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
+++ b/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\git\repository3\MakeMyTrip_Sprint\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEC11D9B-7D99-43E2-9C10-FA42B6F6FCE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAB4D88-78BA-48A8-86D4-4A2A46583EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE859187-6724-4D77-AF72-93B2659ED249}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{AE859187-6724-4D77-AF72-93B2659ED249}"/>
   </bookViews>
   <sheets>
     <sheet name="Train" sheetId="1" r:id="rId1"/>
-    <sheet name="Cab" sheetId="2" r:id="rId2"/>
-    <sheet name="HP" sheetId="3" r:id="rId3"/>
-    <sheet name="HPTravellerDetail" sheetId="4" r:id="rId4"/>
-    <sheet name="FlightTracker" sheetId="5" r:id="rId5"/>
+    <sheet name="HP" sheetId="3" r:id="rId2"/>
+    <sheet name="Cab" sheetId="6" r:id="rId3"/>
+    <sheet name="Hotel" sheetId="7" r:id="rId4"/>
+    <sheet name="HPTravellerDetail" sheetId="4" r:id="rId5"/>
+    <sheet name="FlightTracker" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="70">
   <si>
     <t>Source</t>
   </si>
@@ -203,13 +204,58 @@
   </si>
   <si>
     <t>12 PM - 6 PM</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Renuka</t>
+  </si>
+  <si>
+    <t>renuka@gmail.com</t>
+  </si>
+  <si>
+    <t>Priya</t>
+  </si>
+  <si>
+    <t>priya@gmail.com</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>arjun@gmail.com</t>
+  </si>
+  <si>
+    <t>Testcase</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>checkin</t>
+  </si>
+  <si>
+    <t>checkout</t>
+  </si>
+  <si>
+    <t>Bangalore</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,6 +267,29 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -243,10 +312,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -257,11 +327,22 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -646,56 +727,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D92E795-A112-4BD0-ACD4-4D3B28C5C15E}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="4"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5B765DA-3D68-46F8-B1D7-1969A16A579E}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -889,7 +920,132 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03208968-6F2C-4602-B3C5-97ADEE1F8FB5}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="5">
+        <v>9876543210</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C3" s="5">
+        <v>9123456789</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="5">
+        <v>9988776655</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="mailto:renuka@gmail.com" xr:uid="{54213B79-B13F-40F0-B5A3-E71C2F1132FB}"/>
+    <hyperlink ref="B3" r:id="rId2" display="mailto:priya@gmail.com" xr:uid="{C58FE052-3AF8-41B4-9288-70F4AD9F221C}"/>
+    <hyperlink ref="B4" r:id="rId3" display="mailto:arjun@gmail.com" xr:uid="{2ACA7ECF-74F4-4E0A-8104-F15A14D9B7B2}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B44F61ED-9C7C-4F28-B666-028E33F0E357}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="8">
+        <v>11</v>
+      </c>
+      <c r="D2" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="8">
+        <v>12</v>
+      </c>
+      <c r="D3" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="8">
+        <v>13</v>
+      </c>
+      <c r="D4" s="8">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59C724BA-46F4-49CF-9C0B-74B250AC3507}">
   <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -968,7 +1124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB0F3389-4DA8-42F8-AB80-41CCE53DAB56}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -985,28 +1141,28 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="4"/>
+      <c r="C2" s="7"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="4"/>
+      <c r="C3" s="7"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
Commiting the report updates
</commit_message>
<xml_diff>
--- a/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
+++ b/MakeMyTrip_Sprint/src/test/resources/testdata/MakeMyTripExcelData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\git\repository3\MakeMyTrip_Sprint\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haris\git\MakeMyTrip_Sprint\MakeMyTrip_Sprint\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAB4D88-78BA-48A8-86D4-4A2A46583EE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A25464-4A93-42CA-B5CD-2441DE1589F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{AE859187-6724-4D77-AF72-93B2659ED249}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE859187-6724-4D77-AF72-93B2659ED249}"/>
   </bookViews>
   <sheets>
     <sheet name="Train" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="95">
   <si>
     <t>Source</t>
   </si>
@@ -194,9 +194,6 @@
     <t>Jul</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
     <t>Salem</t>
   </si>
   <si>
@@ -249,6 +246,84 @@
   </si>
   <si>
     <t>Mumbai</t>
+  </si>
+  <si>
+    <t>Coimbatore</t>
+  </si>
+  <si>
+    <t>June</t>
+  </si>
+  <si>
+    <t>AC 3 Tier</t>
+  </si>
+  <si>
+    <t>6 PM - 12 AM</t>
+  </si>
+  <si>
+    <t>Express</t>
+  </si>
+  <si>
+    <t>July</t>
+  </si>
+  <si>
+    <t>Chair Car</t>
+  </si>
+  <si>
+    <t>Madurai</t>
+  </si>
+  <si>
+    <t>Trichy</t>
+  </si>
+  <si>
+    <t>August</t>
+  </si>
+  <si>
+    <t>12 AM - 6 AM</t>
+  </si>
+  <si>
+    <t>Passenger</t>
+  </si>
+  <si>
+    <t>Erode</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <t>Second Sitting</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>AC 2 Tier</t>
+  </si>
+  <si>
+    <t>November</t>
+  </si>
+  <si>
+    <t>Mail</t>
+  </si>
+  <si>
+    <t>December</t>
+  </si>
+  <si>
+    <t>Intercity</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>AC First Class</t>
+  </si>
+  <si>
+    <t>April</t>
   </si>
 </sst>
 </file>
@@ -316,15 +391,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -336,10 +408,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -655,10 +727,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42C36B47-3263-42EC-9348-FE092B284D98}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="9.109375" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" customWidth="1"/>
+    <col min="2" max="2" width="11.88671875" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" customWidth="1"/>
     <col min="6" max="6" width="21.5546875" customWidth="1"/>
     <col min="7" max="7" width="20.109375" customWidth="1"/>
     <col min="8" max="8" width="15.88671875" customWidth="1"/>
@@ -690,35 +765,321 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>51</v>
+      <c r="D2" s="2">
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>54</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="2">
+        <v>12</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="2">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D5" s="2">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" s="2">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" s="2">
+        <v>27</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="2">
+        <v>14</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D9" s="2">
+        <v>3</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D10" s="2">
+        <v>21</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11" s="2">
+        <v>9</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D12" s="2">
+        <v>16</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" s="2">
+        <v>28</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:G19" xr:uid="{54DE1FC2-7873-4FF0-9E14-1AE5979033BC}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F14:G19" xr:uid="{54DE1FC2-7873-4FF0-9E14-1AE5979033BC}">
       <formula1>"12am - 6am,6am - 12pm,12pm - 6pm,6pm - 12am"</formula1>
     </dataValidation>
   </dataValidations>
@@ -926,46 +1287,46 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="B2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="4">
+        <v>9876543210</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="5">
-        <v>9876543210</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="B3" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C3" s="4">
+        <v>9123456789</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C3" s="5">
-        <v>9123456789</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>9988776655</v>
       </c>
     </row>
@@ -985,58 +1346,58 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="6">
+        <v>11</v>
+      </c>
+      <c r="D2" s="6">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="8">
-        <v>11</v>
-      </c>
-      <c r="D2" s="8">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="6">
+        <v>12</v>
+      </c>
+      <c r="D3" s="6">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C3" s="8">
-        <v>12</v>
-      </c>
-      <c r="D3" s="8">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4" s="8">
+      <c r="C4" s="6">
         <v>13</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="6">
         <v>16</v>
       </c>
     </row>

</xml_diff>